<commit_message>
Added screenshot to the extent report
</commit_message>
<xml_diff>
--- a/src/test/resources/testResources/LoginInfo.xlsx
+++ b/src/test/resources/testResources/LoginInfo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/85ca7b966e090d8a/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sharath\eclipse-workspace\MiniFrameWorkProject\src\test\resources\testResources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A38B530E-6472-4EE3-BC04-9678102DC6DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF0312C-45D3-47E7-A19D-9A117C40DF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{03CCC5CA-81F5-4729-9AA5-8600DAAC7012}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
   <si>
     <t>Username</t>
   </si>
@@ -52,6 +52,18 @@
   </si>
   <si>
     <t>Test@123</t>
+  </si>
+  <si>
+    <t>user1780655706479@gmail.com</t>
+  </si>
+  <si>
+    <t>user1780662301235@gmail.com</t>
+  </si>
+  <si>
+    <t>user1781004104419@gmail.com</t>
+  </si>
+  <si>
+    <t>user1781009565603@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -404,8 +416,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B2EB934-9469-4E83-AC37-2F871E0CD9DF}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="28.109375"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s" s="0">
@@ -423,11 +438,43 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s" s="0">
         <v>4</v>
       </c>
       <c r="B3" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s" s="0">
         <v>5</v>
       </c>
     </row>

</xml_diff>